<commit_message>
first simmulations euler prueba
</commit_message>
<xml_diff>
--- a/6node_spain/output_a.xlsx
+++ b/6node_spain/output_a.xlsx
@@ -489,13 +489,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1.473962980448705</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8700077517613194</v>
+        <v>0.8130081300813008</v>
       </c>
     </row>
     <row r="4">
@@ -514,13 +514,13 @@
         <v>0</v>
       </c>
       <c r="E4" t="n">
-        <v>0.656378759174014</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>0.2263192170913441</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -533,10 +533,10 @@
         <v>0</v>
       </c>
       <c r="C5" t="n">
-        <v>1.473962980448705</v>
+        <v>0</v>
       </c>
       <c r="D5" t="n">
-        <v>0.656378759174014</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -545,7 +545,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3797202509695052</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -570,7 +570,7 @@
         <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>0.1243543496159273</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7">
@@ -583,16 +583,16 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8700077517613194</v>
+        <v>0.8130081300813008</v>
       </c>
       <c r="D7" t="n">
-        <v>0.2263192170913441</v>
+        <v>0</v>
       </c>
       <c r="E7" t="n">
-        <v>0.3797202509695052</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>0.1243543496159273</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
add euler 40k sim
</commit_message>
<xml_diff>
--- a/6node_spain/output_a.xlsx
+++ b/6node_spain/output_a.xlsx
@@ -495,7 +495,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0.8130081300813008</v>
+        <v>2.345878066070536</v>
       </c>
     </row>
     <row r="4">
@@ -583,7 +583,7 @@
         <v>0</v>
       </c>
       <c r="C7" t="n">
-        <v>0.8130081300813008</v>
+        <v>2.345878066070536</v>
       </c>
       <c r="D7" t="n">
         <v>0</v>

</xml_diff>